<commit_message>
Enhance Google Sheets integration with bidirectional data synchronization
Implement bidirectional data synchronization for Google Sheets, allowing both pushing app data to the sheet and pulling sheet changes back into the application. This also includes UI updates for new import functionality and improved quick login user data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 99ec330d-0375-46ca-a20e-c13b3d7787a9
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/pCexr2j
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-13.xlsx
+++ b/backups/proposal-log-2026-03-13.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>HK</t>
+  </si>
+  <si>
+    <t>3000</t>
   </si>
   <si>
     <t>2027-02-01</t>
@@ -748,24 +751,24 @@
         <v>19</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="J5" t="s">
         <v>20</v>
       </c>
       <c r="K5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
         <v>14</v>
@@ -774,7 +777,7 @@
         <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
@@ -792,10 +795,10 @@
         <v>20</v>
       </c>
       <c r="K6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="L6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix HomePage HUD: server-side acknowledgements, estimator filtering, live sync, past-due visibility
- Switched HUD acknowledgement tracking from localStorage to server-side API
  (GET/POST /api/proposal-log/acknowledgements)
- HUD now shows only bids assigned to the logged-in estimator (strict match on nbsEstimator)
- Fixed bizDaysUntil() to return accurate negative business day counts for past-due bids
- Replaced localStorage polling with direct server fetch every 10s + refetch on window focus
- Past-due bids now appear correctly in the HUD instead of being filtered out
- Removed all stale localStorage-based caching (persistAcknowledged, ACK_STORAGE_KEY, etc.)
- Session plan tasks T001-T006 all verified complete
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-13.xlsx
+++ b/backups/proposal-log-2026-03-13.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="49">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -134,9 +134,6 @@
   </si>
   <si>
     <t>2026-03-24</t>
-  </si>
-  <si>
-    <t>HK</t>
   </si>
   <si>
     <t>3000</t>
@@ -745,30 +742,30 @@
         <v>40</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s">
         <v>19</v>
       </c>
       <c r="I5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J5" t="s">
         <v>20</v>
       </c>
       <c r="K5" t="s">
+        <v>42</v>
+      </c>
+      <c r="L5" t="s">
         <v>43</v>
-      </c>
-      <c r="L5" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" t="s">
         <v>45</v>
-      </c>
-      <c r="B6" t="s">
-        <v>46</v>
       </c>
       <c r="C6" t="s">
         <v>14</v>
@@ -777,13 +774,13 @@
         <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
       </c>
       <c r="G6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H6" t="s">
         <v>19</v>
@@ -795,10 +792,10 @@
         <v>20</v>
       </c>
       <c r="K6" t="s">
+        <v>47</v>
+      </c>
+      <c r="L6" t="s">
         <v>48</v>
-      </c>
-      <c r="L6" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Align proposal log icons and fix animation for acknowledgments
Update CSS to ensure consistent grid alignment for icons across proposal log sections. Modify the acknowledgment logic to use stable IDs and defer API calls until after animations complete, preventing visual glitches.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: d97c3081-6f17-4f71-950c-f1dbea273634
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/488UOpv
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-13.xlsx
+++ b/backups/proposal-log-2026-03-13.xlsx
@@ -97,61 +97,61 @@
     <t>2026-03-18</t>
   </si>
   <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-11-30</t>
+  </si>
+  <si>
+    <t>26-0026</t>
+  </si>
+  <si>
+    <t>Morgan Stanley Tacoma Interior Improvements</t>
+  </si>
+  <si>
+    <t>Washington (SEA)</t>
+  </si>
+  <si>
+    <t>2026-03-13</t>
+  </si>
+  <si>
+    <t>2026-03-26</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>2026-07-06</t>
+  </si>
+  <si>
+    <t>26-0027</t>
+  </si>
+  <si>
+    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>3000</t>
+  </si>
+  <si>
+    <t>2027-02-01</t>
+  </si>
+  <si>
+    <t>2028-02-29</t>
+  </si>
+  <si>
+    <t>26-0028</t>
+  </si>
+  <si>
+    <t>Burbank Cargo &amp; GSE Buildout</t>
+  </si>
+  <si>
+    <t>2026-03-12</t>
+  </si>
+  <si>
     <t>GM</t>
-  </si>
-  <si>
-    <t>2026-04-01</t>
-  </si>
-  <si>
-    <t>2026-11-30</t>
-  </si>
-  <si>
-    <t>26-0026</t>
-  </si>
-  <si>
-    <t>Morgan Stanley Tacoma Interior Improvements</t>
-  </si>
-  <si>
-    <t>Washington (SEA)</t>
-  </si>
-  <si>
-    <t>2026-03-13</t>
-  </si>
-  <si>
-    <t>2026-03-26</t>
-  </si>
-  <si>
-    <t>2026-05-07</t>
-  </si>
-  <si>
-    <t>2026-07-06</t>
-  </si>
-  <si>
-    <t>26-0027</t>
-  </si>
-  <si>
-    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS</t>
-  </si>
-  <si>
-    <t>2026-03-24</t>
-  </si>
-  <si>
-    <t>3000</t>
-  </si>
-  <si>
-    <t>2027-02-01</t>
-  </si>
-  <si>
-    <t>2028-02-29</t>
-  </si>
-  <si>
-    <t>26-0028</t>
-  </si>
-  <si>
-    <t>Burbank Cargo &amp; GSE Buildout</t>
-  </si>
-  <si>
-    <t>2026-03-12</t>
   </si>
   <si>
     <t>2026-05-01</t>
@@ -666,7 +666,7 @@
         <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H3" t="s">
         <v>19</v>
@@ -678,33 +678,33 @@
         <v>20</v>
       </c>
       <c r="K3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" t="s">
         <v>29</v>
-      </c>
-      <c r="L3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>33</v>
       </c>
       <c r="D4" t="s">
         <v>25</v>
       </c>
       <c r="E4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
         <v>34</v>
       </c>
-      <c r="F4" t="s">
-        <v>35</v>
-      </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H4" t="s">
         <v>19</v>
@@ -716,18 +716,18 @@
         <v>20</v>
       </c>
       <c r="K4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" t="s">
         <v>36</v>
-      </c>
-      <c r="L4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
         <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>14</v>
@@ -736,36 +736,36 @@
         <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H5" t="s">
         <v>19</v>
       </c>
       <c r="I5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J5" t="s">
         <v>20</v>
       </c>
       <c r="K5" t="s">
+        <v>41</v>
+      </c>
+      <c r="L5" t="s">
         <v>42</v>
-      </c>
-      <c r="L5" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s">
         <v>44</v>
-      </c>
-      <c r="B6" t="s">
-        <v>45</v>
       </c>
       <c r="C6" t="s">
         <v>14</v>
@@ -774,13 +774,13 @@
         <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
       </c>
       <c r="G6" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="H6" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Improve proposal status updates and filtering logic
Automatically update proposal status to "Submitted" when a proposalTotal is entered, and revert to "Estimating" when cleared. Update homepage to only display "Estimating" bids. Synchronize status changes to the server.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e74a6f2c-4573-4ac4-acdb-7af1495594f8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/488UOpv
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-13.xlsx
+++ b/backups/proposal-log-2026-03-13.xlsx
@@ -97,6 +97,9 @@
     <t>2026-03-18</t>
   </si>
   <si>
+    <t>HK</t>
+  </si>
+  <si>
     <t>2026-04-01</t>
   </si>
   <si>
@@ -149,9 +152,6 @@
   </si>
   <si>
     <t>2026-03-12</t>
-  </si>
-  <si>
-    <t>GM</t>
   </si>
   <si>
     <t>2026-05-01</t>
@@ -666,7 +666,7 @@
         <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H3" t="s">
         <v>19</v>
@@ -678,33 +678,33 @@
         <v>20</v>
       </c>
       <c r="K3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
         <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
         <v>19</v>
@@ -716,18 +716,18 @@
         <v>20</v>
       </c>
       <c r="K4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>14</v>
@@ -736,36 +736,36 @@
         <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G5" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s">
         <v>19</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J5" t="s">
         <v>20</v>
       </c>
       <c r="K5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
         <v>14</v>
@@ -774,13 +774,13 @@
         <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
       </c>
       <c r="G6" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="H6" t="s">
         <v>19</v>

</xml_diff>